<commit_message>
Bug fix in unrestrained
</commit_message>
<xml_diff>
--- a/UB-2.xlsx
+++ b/UB-2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/twalha/Documents/GitHub/g6-analysis-tool/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98E03722-B37D-5A4C-9A81-A6F032BD8E25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55A92AA4-4F38-2E45-9BDF-B9203209AFD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Steel Section Properties Data" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="73">
   <si>
     <t>Section Designation</t>
   </si>
@@ -249,6 +249,9 @@
   </si>
   <si>
     <t>457x191x161 +</t>
+  </si>
+  <si>
+    <t>b (mm)</t>
   </si>
 </sst>
 </file>
@@ -519,10 +522,10 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:R55"/>
+  <dimension ref="A1:S55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <sheetData>
-    <row r="1" spans="1:18" ht="13" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -577,8 +580,11 @@
       <c r="R1" s="1" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" ht="13" x14ac:dyDescent="0.15">
+      <c r="S1" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A2" s="2" t="s">
         <v>17</v>
       </c>
@@ -621,8 +627,11 @@
       <c r="R2" s="2">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:18" ht="13" x14ac:dyDescent="0.15">
+      <c r="S2" s="2">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A3" s="2" t="s">
         <v>18</v>
       </c>
@@ -665,8 +674,11 @@
       <c r="R3" s="2">
         <v>7</v>
       </c>
-    </row>
-    <row r="4" spans="1:18" ht="13" x14ac:dyDescent="0.15">
+      <c r="S3" s="2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -709,8 +721,11 @@
       <c r="R4" s="2">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="1:18" ht="13" x14ac:dyDescent="0.15">
+      <c r="S4" s="2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -753,8 +768,11 @@
       <c r="R5" s="2">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" spans="1:18" ht="13" x14ac:dyDescent="0.15">
+      <c r="S5" s="2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A6" s="2" t="s">
         <v>21</v>
       </c>
@@ -797,8 +815,11 @@
       <c r="R6" s="2">
         <v>9</v>
       </c>
-    </row>
-    <row r="7" spans="1:18" ht="13" x14ac:dyDescent="0.15">
+      <c r="S6" s="2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A7" s="2" t="s">
         <v>22</v>
       </c>
@@ -841,8 +862,11 @@
       <c r="R7" s="2">
         <v>9</v>
       </c>
-    </row>
-    <row r="8" spans="1:18" ht="13" x14ac:dyDescent="0.15">
+      <c r="S7" s="2">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A8" s="2" t="s">
         <v>23</v>
       </c>
@@ -885,8 +909,11 @@
       <c r="R8" s="2">
         <v>12</v>
       </c>
-    </row>
-    <row r="9" spans="1:18" ht="13" x14ac:dyDescent="0.15">
+      <c r="S8" s="2">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A9" s="2" t="s">
         <v>24</v>
       </c>
@@ -929,8 +956,11 @@
       <c r="R9" s="2">
         <v>12</v>
       </c>
-    </row>
-    <row r="10" spans="1:18" ht="13" x14ac:dyDescent="0.15">
+      <c r="S9" s="2">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A10" s="2" t="s">
         <v>25</v>
       </c>
@@ -973,8 +1003,11 @@
       <c r="R10" s="2">
         <v>15</v>
       </c>
-    </row>
-    <row r="11" spans="1:18" ht="13" x14ac:dyDescent="0.15">
+      <c r="S10" s="2">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A11" s="2" t="s">
         <v>26</v>
       </c>
@@ -1017,8 +1050,11 @@
       <c r="R11" s="2">
         <v>15</v>
       </c>
-    </row>
-    <row r="12" spans="1:18" ht="13" x14ac:dyDescent="0.15">
+      <c r="S11" s="2">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A12" s="2" t="s">
         <v>27</v>
       </c>
@@ -1061,8 +1097,11 @@
       <c r="R12" s="2">
         <v>15</v>
       </c>
-    </row>
-    <row r="13" spans="1:18" ht="13" x14ac:dyDescent="0.15">
+      <c r="S12" s="2">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A13" s="2" t="s">
         <v>28</v>
       </c>
@@ -1105,8 +1144,11 @@
       <c r="R13" s="2">
         <v>18</v>
       </c>
-    </row>
-    <row r="14" spans="1:18" ht="13" x14ac:dyDescent="0.15">
+      <c r="S13" s="2">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A14" s="2" t="s">
         <v>29</v>
       </c>
@@ -1149,8 +1191,11 @@
       <c r="R14" s="2">
         <v>18</v>
       </c>
-    </row>
-    <row r="15" spans="1:18" ht="13" x14ac:dyDescent="0.15">
+      <c r="S14" s="2">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A15" s="2" t="s">
         <v>30</v>
       </c>
@@ -1193,8 +1238,11 @@
       <c r="R15" s="2">
         <v>21</v>
       </c>
-    </row>
-    <row r="16" spans="1:18" ht="13" x14ac:dyDescent="0.15">
+      <c r="S15" s="2">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A16" s="2" t="s">
         <v>31</v>
       </c>
@@ -1237,8 +1285,11 @@
       <c r="R16" s="2">
         <v>21</v>
       </c>
-    </row>
-    <row r="17" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S16" s="2">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A17" s="1" t="s">
         <v>33</v>
       </c>
@@ -1290,8 +1341,11 @@
       <c r="Q17">
         <v>8.5</v>
       </c>
-    </row>
-    <row r="18" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S17">
+        <v>125.4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A18" s="1" t="s">
         <v>34</v>
       </c>
@@ -1343,8 +1397,11 @@
       <c r="Q18">
         <v>8.6</v>
       </c>
-    </row>
-    <row r="19" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S18">
+        <v>141.80000000000001</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A19" s="1" t="s">
         <v>35</v>
       </c>
@@ -1396,8 +1453,11 @@
       <c r="Q19">
         <v>10.7</v>
       </c>
-    </row>
-    <row r="20" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S19">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A20" s="1" t="s">
         <v>36</v>
       </c>
@@ -1449,8 +1509,11 @@
       <c r="Q20">
         <v>10.199999999999999</v>
       </c>
-    </row>
-    <row r="21" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S20">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A21" s="1" t="s">
         <v>37</v>
       </c>
@@ -1502,8 +1565,11 @@
       <c r="Q21">
         <v>9.6999999999999993</v>
       </c>
-    </row>
-    <row r="22" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S21">
+        <v>171.1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A22" s="1" t="s">
         <v>38</v>
       </c>
@@ -1555,8 +1621,11 @@
       <c r="Q22">
         <v>11.2</v>
       </c>
-    </row>
-    <row r="23" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S22">
+        <v>142.19999999999999</v>
+      </c>
+    </row>
+    <row r="23" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A23" s="1" t="s">
         <v>39</v>
       </c>
@@ -1608,8 +1677,11 @@
       <c r="Q23">
         <v>11.8</v>
       </c>
-    </row>
-    <row r="24" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S23">
+        <v>165.7</v>
+      </c>
+    </row>
+    <row r="24" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A24" s="1" t="s">
         <v>40</v>
       </c>
@@ -1661,8 +1733,11 @@
       <c r="Q24">
         <v>11.5</v>
       </c>
-    </row>
-    <row r="25" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S24">
+        <v>171.5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A25" s="1" t="s">
         <v>41</v>
       </c>
@@ -1714,8 +1789,11 @@
       <c r="Q25">
         <v>10.9</v>
       </c>
-    </row>
-    <row r="26" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S25">
+        <v>152.4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A26" s="1" t="s">
         <v>42</v>
       </c>
@@ -1767,8 +1845,11 @@
       <c r="Q26">
         <v>12.9</v>
       </c>
-    </row>
-    <row r="27" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S26">
+        <v>143.30000000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A27" s="1" t="s">
         <v>43</v>
       </c>
@@ -1820,8 +1901,11 @@
       <c r="Q27">
         <v>13.7</v>
       </c>
-    </row>
-    <row r="28" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S27">
+        <v>166.9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A28" s="1" t="s">
         <v>44</v>
       </c>
@@ -1873,8 +1957,11 @@
       <c r="Q28">
         <v>10.9</v>
       </c>
-    </row>
-    <row r="29" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S28">
+        <v>177.7</v>
+      </c>
+    </row>
+    <row r="29" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A29" s="1" t="s">
         <v>45</v>
       </c>
@@ -1926,8 +2013,11 @@
       <c r="Q29">
         <v>13</v>
       </c>
-    </row>
-    <row r="30" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S29">
+        <v>172.2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A30" s="1" t="s">
         <v>46</v>
       </c>
@@ -1979,8 +2069,11 @@
       <c r="Q30">
         <v>13.3</v>
       </c>
-    </row>
-    <row r="31" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S30">
+        <v>152.9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A31" s="1" t="s">
         <v>47</v>
       </c>
@@ -2032,8 +2125,11 @@
       <c r="Q31">
         <v>12.8</v>
       </c>
-    </row>
-    <row r="32" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S31">
+        <v>177.9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A32" s="1" t="s">
         <v>48</v>
       </c>
@@ -2085,8 +2181,11 @@
       <c r="Q32">
         <v>11.4</v>
       </c>
-    </row>
-    <row r="33" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S32">
+        <v>165.1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A33" s="1" t="s">
         <v>49</v>
       </c>
@@ -2138,8 +2237,11 @@
       <c r="Q33">
         <v>12.7</v>
       </c>
-    </row>
-    <row r="34" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S33">
+        <v>189.9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A34" s="1" t="s">
         <v>50</v>
       </c>
@@ -2191,8 +2293,11 @@
       <c r="Q34">
         <v>14.3</v>
       </c>
-    </row>
-    <row r="35" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S34">
+        <v>178.5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A35" s="1" t="s">
         <v>51</v>
       </c>
@@ -2244,8 +2349,11 @@
       <c r="Q35">
         <v>15.7</v>
       </c>
-    </row>
-    <row r="36" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S35">
+        <v>173.2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A36" s="1" t="s">
         <v>52</v>
       </c>
@@ -2297,8 +2405,11 @@
       <c r="Q36">
         <v>15</v>
       </c>
-    </row>
-    <row r="37" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S36">
+        <v>153.80000000000001</v>
+      </c>
+    </row>
+    <row r="37" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A37" s="1" t="s">
         <v>53</v>
       </c>
@@ -2350,8 +2461,11 @@
       <c r="Q37">
         <v>17</v>
       </c>
-    </row>
-    <row r="38" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S37">
+        <v>154.4</v>
+      </c>
+    </row>
+    <row r="38" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A38" s="1" t="s">
         <v>54</v>
       </c>
@@ -2403,8 +2517,11 @@
       <c r="Q38">
         <v>16</v>
       </c>
-    </row>
-    <row r="39" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S38">
+        <v>179.5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A39" s="1" t="s">
         <v>55</v>
       </c>
@@ -2456,8 +2573,11 @@
       <c r="Q39">
         <v>14.5</v>
       </c>
-    </row>
-    <row r="40" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S39">
+        <v>190.4</v>
+      </c>
+    </row>
+    <row r="40" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A40" s="1" t="s">
         <v>56</v>
       </c>
@@ -2509,8 +2629,11 @@
       <c r="Q40">
         <v>13.6</v>
       </c>
-    </row>
-    <row r="41" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S40">
+        <v>165.9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A41" s="1" t="s">
         <v>57</v>
       </c>
@@ -2562,8 +2685,11 @@
       <c r="Q41">
         <v>16</v>
       </c>
-    </row>
-    <row r="42" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S41">
+        <v>191.3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A42" s="1" t="s">
         <v>58</v>
       </c>
@@ -2615,8 +2741,11 @@
       <c r="Q42">
         <v>13.2</v>
       </c>
-    </row>
-    <row r="43" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S42">
+        <v>208.8</v>
+      </c>
+    </row>
+    <row r="43" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A43" s="1" t="s">
         <v>59</v>
       </c>
@@ -2668,8 +2797,11 @@
       <c r="Q43">
         <v>18.899999999999999</v>
       </c>
-    </row>
-    <row r="44" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S43">
+        <v>155.30000000000001</v>
+      </c>
+    </row>
+    <row r="44" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A44" s="1" t="s">
         <v>60</v>
       </c>
@@ -2721,8 +2853,11 @@
       <c r="Q44">
         <v>16.5</v>
       </c>
-    </row>
-    <row r="45" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S44">
+        <v>166.5</v>
+      </c>
+    </row>
+    <row r="45" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A45" s="1" t="s">
         <v>61</v>
       </c>
@@ -2774,8 +2909,11 @@
       <c r="Q45">
         <v>18.2</v>
       </c>
-    </row>
-    <row r="46" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S45">
+        <v>181.9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A46" s="1" t="s">
         <v>62</v>
       </c>
@@ -2827,8 +2965,11 @@
       <c r="Q46">
         <v>17.7</v>
       </c>
-    </row>
-    <row r="47" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S46">
+        <v>191.9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A47" s="1" t="s">
         <v>63</v>
       </c>
@@ -2880,8 +3021,11 @@
       <c r="Q47">
         <v>15.6</v>
       </c>
-    </row>
-    <row r="48" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S47">
+        <v>209.3</v>
+      </c>
+    </row>
+    <row r="48" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A48" s="1" t="s">
         <v>64</v>
       </c>
@@ -2933,8 +3077,11 @@
       <c r="Q48">
         <v>19.600000000000001</v>
       </c>
-    </row>
-    <row r="49" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S48">
+        <v>192.8</v>
+      </c>
+    </row>
+    <row r="49" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A49" s="1" t="s">
         <v>65</v>
       </c>
@@ -2986,8 +3133,11 @@
       <c r="Q49">
         <v>17.399999999999999</v>
       </c>
-    </row>
-    <row r="50" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S49">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="50" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A50" s="1" t="s">
         <v>66</v>
       </c>
@@ -3039,8 +3189,11 @@
       <c r="Q50">
         <v>20.6</v>
       </c>
-    </row>
-    <row r="51" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S50">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="51" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A51" s="1" t="s">
         <v>67</v>
       </c>
@@ -3092,8 +3245,11 @@
       <c r="Q51">
         <v>18.8</v>
       </c>
-    </row>
-    <row r="52" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S51">
+        <v>210.8</v>
+      </c>
+    </row>
+    <row r="52" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A52" s="1" t="s">
         <v>68</v>
       </c>
@@ -3145,8 +3301,11 @@
       <c r="Q52">
         <v>21.3</v>
       </c>
-    </row>
-    <row r="53" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S52">
+        <v>211.9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A53" s="1" t="s">
         <v>69</v>
       </c>
@@ -3198,8 +3357,11 @@
       <c r="Q53">
         <v>26.3</v>
       </c>
-    </row>
-    <row r="54" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S53">
+        <v>196.7</v>
+      </c>
+    </row>
+    <row r="54" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A54" s="1" t="s">
         <v>70</v>
       </c>
@@ -3251,8 +3413,11 @@
       <c r="Q54">
         <v>23.6</v>
       </c>
-    </row>
-    <row r="55" spans="1:17" ht="13" x14ac:dyDescent="0.15">
+      <c r="S54">
+        <v>213.9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:19" ht="13" x14ac:dyDescent="0.15">
       <c r="A55" s="1" t="s">
         <v>71</v>
       </c>
@@ -3303,6 +3468,9 @@
       </c>
       <c r="Q55">
         <v>32</v>
+      </c>
+      <c r="S55">
+        <v>199.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>